<commit_message>
W01 D2: restage the missing-discount trap on the share of orders with a discount
Read as zero, 50.0 percent of Q2's orders (43 of 86) carry a discount and
Marketing extends the monsoon discount to the other half. The check splits the
43 into 17 recorded zeros and 26 blanks; the fix treats a blank as unknown:
71.7 percent of the 60 recorded, a range of 50.0 to 80.2 percent. Carried
through notebook 02, the morning deck S22 to S24, round 2 items 5 and 7, the
study notes, the day sheet, the simulator, the workbook's Discount tab and the
board work. The Kahoot item uses invented counts, and the Kahoot is cut to the
standard's eight by dropping the first-move item.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NDq7Sv6UNg6oqbgZGtNeM1
</commit_message>
<xml_diff>
--- a/content/W01/D2/demos/C2_W01_D02_decision_tool_STUDENT.xlsx
+++ b/content/W01/D2/demos/C2_W01_D02_decision_tool_STUDENT.xlsx
@@ -22,7 +22,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+  </numFmts>
   <fonts count="6">
     <font>
       <name val="Calibri"/>
@@ -103,7 +105,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -117,6 +119,7 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1004,14 +1007,14 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Discount recorded, total (Rs)</t>
+          <t>Orders with a discount above Rs 0</t>
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>2400</v>
+        <v>24</v>
       </c>
       <c r="C7" s="5" t="n">
-        <v>2250</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8">
@@ -1037,14 +1040,14 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Per order, absent read as zero</t>
-        </is>
-      </c>
-      <c r="B11">
+          <t>Share with a discount, absent read as zero</t>
+        </is>
+      </c>
+      <c r="B11" s="9">
         <f>B7/B5</f>
         <v/>
       </c>
-      <c r="C11">
+      <c r="C11" s="9">
         <f>C7/C5</f>
         <v/>
       </c>
@@ -1052,14 +1055,14 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Per order, where recorded</t>
-        </is>
-      </c>
-      <c r="B12">
+          <t>Share with a discount, where recorded</t>
+        </is>
+      </c>
+      <c r="B12" s="9">
         <f>B7/B6</f>
         <v/>
       </c>
-      <c r="C12">
+      <c r="C12" s="9">
         <f>C7/C5</f>
         <v/>
       </c>
@@ -1067,22 +1070,37 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>Share at most, every blank discounted</t>
+        </is>
+      </c>
+      <c r="B13" s="9">
+        <f>(B7+B5-B6)/B5</f>
+        <v/>
+      </c>
+      <c r="C13" s="9">
+        <f>(C7+C5-C6)/C5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>The most the branch could move (Rs)</t>
         </is>
       </c>
-      <c r="C13">
+      <c r="C14">
         <f>B8*C5</f>
         <v/>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>The check</t>
         </is>
       </c>
-      <c r="B14" s="2">
-        <f>IF(AND(ABS(B12*B6-B7)&lt;0.5,ABS(C12*C6-C7)&lt;0.5),"The where-recorded averages multiply back to the recorded totals.","A where-recorded average does not multiply back to its recorded total: it divides by every order. Fix it first.")</f>
+      <c r="B15" s="2">
+        <f>IF(AND(ABS(B12*B6-B7)&lt;0.5,ABS(C12*C6-C7)&lt;0.5),"The where-recorded shares multiply back to the orders with a discount.","A where-recorded share does not multiply back to its orders with a discount: it divides by every order. Fix it first.")</f>
         <v/>
       </c>
     </row>
@@ -1105,7 +1123,7 @@
         </is>
       </c>
       <c r="B18" s="8">
-        <f>IF(OR(ABS(B12*B6-B7)&gt;=0.5,ABS(C12*C6-C7)&gt;=0.5),"Fix the where-recorded average before choosing a default.",IF(B16="read absent as zero","Refuse the zero default: an absent discount is unknown, so the total is a floor; choose a default and write down why.",IF(B16="report where recorded","Report the discount where recorded, "&amp;IF(B12&lt;0,"-","")&amp;"Rs "&amp;IF(ROUND(ABS(B12),0)&gt;=10000000,INT(ROUND(ABS(B12),0)/10000000)&amp;","&amp;TEXT(INT(MOD(ROUND(ABS(B12),0),10000000)/100000),"00")&amp;","&amp;TEXT(INT(MOD(ROUND(ABS(B12),0),100000)/1000),"00")&amp;","&amp;TEXT(MOD(ROUND(ABS(B12),0),1000),"000"),IF(ROUND(ABS(B12),0)&gt;=100000,INT(ROUND(ABS(B12),0)/100000)&amp;","&amp;TEXT(INT(MOD(ROUND(ABS(B12),0),100000)/1000),"00")&amp;","&amp;TEXT(MOD(ROUND(ABS(B12),0),1000),"000"),IF(ROUND(ABS(B12),0)&gt;=1000,INT(ROUND(ABS(B12),0)/1000)&amp;","&amp;TEXT(MOD(ROUND(ABS(B12),0),1000),"000"),ROUND(ABS(B12),0)&amp;"")))&amp;" to "&amp;IF(C12&lt;0,"-","")&amp;"Rs "&amp;IF(ROUND(ABS(C12),0)&gt;=10000000,INT(ROUND(ABS(C12),0)/10000000)&amp;","&amp;TEXT(INT(MOD(ROUND(ABS(C12),0),10000000)/100000),"00")&amp;","&amp;TEXT(INT(MOD(ROUND(ABS(C12),0),100000)/1000),"00")&amp;","&amp;TEXT(MOD(ROUND(ABS(C12),0),1000),"000"),IF(ROUND(ABS(C12),0)&gt;=100000,INT(ROUND(ABS(C12),0)/100000)&amp;","&amp;TEXT(INT(MOD(ROUND(ABS(C12),0),100000)/1000),"00")&amp;","&amp;TEXT(MOD(ROUND(ABS(C12),0),1000),"000"),IF(ROUND(ABS(C12),0)&gt;=1000,INT(ROUND(ABS(C12),0)/1000)&amp;","&amp;TEXT(MOD(ROUND(ABS(C12),0),1000),"000"),ROUND(ABS(C12),0)&amp;"")))&amp;" an order, with the orders that lack the field reported separately.","The discount branch is at most "&amp;IF(C13&lt;0,"-","")&amp;"Rs "&amp;IF(ROUND(ABS(C13),0)&gt;=10000000,INT(ROUND(ABS(C13),0)/10000000)&amp;","&amp;TEXT(INT(MOD(ROUND(ABS(C13),0),10000000)/100000),"00")&amp;","&amp;TEXT(INT(MOD(ROUND(ABS(C13),0),100000)/1000),"00")&amp;","&amp;TEXT(MOD(ROUND(ABS(C13),0),1000),"000"),IF(ROUND(ABS(C13),0)&gt;=100000,INT(ROUND(ABS(C13),0)/100000)&amp;","&amp;TEXT(INT(MOD(ROUND(ABS(C13),0),100000)/1000),"00")&amp;","&amp;TEXT(MOD(ROUND(ABS(C13),0),1000),"000"),IF(ROUND(ABS(C13),0)&gt;=1000,INT(ROUND(ABS(C13),0)/1000)&amp;","&amp;TEXT(MOD(ROUND(ABS(C13),0),1000),"000"),ROUND(ABS(C13),0)&amp;"")))&amp;", "&amp;TEXT(100*C13/B9,"0.00")&amp;" percent of the fall, so it did not move revenue.")))</f>
+        <f>IF(OR(ABS(B12*B6-B7)&gt;=0.5,ABS(C12*C6-C7)&gt;=0.5),"Fix the where-recorded share before choosing a default.",IF(B16="read absent as zero","Refuse the zero default: an absent discount is unknown, so the share is a floor; choose a default and write down why.",IF(B16="report where recorded","Report the share where recorded, "&amp;TEXT(B12,"0.0%")&amp;" to "&amp;TEXT(C12,"0.0%")&amp;" of orders, with the orders that lack the field reported separately.","The discount branch is at most "&amp;IF(C14&lt;0,"-","")&amp;"Rs "&amp;IF(ROUND(ABS(C14),0)&gt;=10000000,INT(ROUND(ABS(C14),0)/10000000)&amp;","&amp;TEXT(INT(MOD(ROUND(ABS(C14),0),10000000)/100000),"00")&amp;","&amp;TEXT(INT(MOD(ROUND(ABS(C14),0),100000)/1000),"00")&amp;","&amp;TEXT(MOD(ROUND(ABS(C14),0),1000),"000"),IF(ROUND(ABS(C14),0)&gt;=100000,INT(ROUND(ABS(C14),0)/100000)&amp;","&amp;TEXT(INT(MOD(ROUND(ABS(C14),0),100000)/1000),"00")&amp;","&amp;TEXT(MOD(ROUND(ABS(C14),0),1000),"000"),IF(ROUND(ABS(C14),0)&gt;=1000,INT(ROUND(ABS(C14),0)/1000)&amp;","&amp;TEXT(MOD(ROUND(ABS(C14),0),1000),"000"),ROUND(ABS(C14),0)&amp;"")))&amp;", "&amp;TEXT(100*C14/B9,"0.00")&amp;" percent of the fall, so it did not move revenue.")))</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
W01 D2 notes, day sheet, board work, pre-read, cheat sheet and companion ask their questions; chapter 6's ceiling carries both baselines
The notes open on the day's question and put each chapter under its full question with who needs the
answer, its six smaller questions as subheadings and a closing answer. The day sheet prints the whole
ladder at its top, renumbers every slide range to the rebuilt decks (the room finds the segment at
S52) and states the ceiling as about 4 on the 55 days before the break and 7.0 on the 37 days just
before it. The companion's headings and guided walk ask their questions and its glossary points at
chapters, where it pointed at the retired rounds; the workbook's tab titles ask theirs. The cheat sheet
is rebuilt on one page.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Hb9A6qKwU75M1ZPNLDhr3q
</commit_message>
<xml_diff>
--- a/content/W01/D2/demos/C2_W01_D02_decision_tool_STUDENT.xlsx
+++ b/content/W01/D2/demos/C2_W01_D02_decision_tool_STUDENT.xlsx
@@ -494,7 +494,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Which branch moved: the decision tool</t>
+          <t>Which branch moved from Q1 to Q2, one decision at a time?</t>
         </is>
       </c>
     </row>
@@ -1168,7 +1168,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Weighted or averaged?</t>
+          <t>Should the segments be weighted or averaged?</t>
         </is>
       </c>
     </row>
@@ -1394,7 +1394,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Groups in against groups out</t>
+          <t>Does every group that goes in come back out?</t>
         </is>
       </c>
     </row>
@@ -1618,7 +1618,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>The brief, assembled</t>
+          <t>Is the brief ready to go to Meera?</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
W01 D2 reviewer fixes outside the decks: the notes, day sheet, board work, pre-read, cheat sheet, companion and workbook read with nothing else open
The notes end on the day's own question and its answer, and self-test item 1 names the same weeks
of both quarters with a rate per week beside them. The day sheet asks chapter 4's sixth question in
full and qualifies the season answer. The cheat sheet PDF is rebuilt from its markdown. The
workbook's window verdicts say what to send while a quarter is open, and the recalc manifest
expects the new text.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Hb9A6qKwU75M1ZPNLDhr3q
</commit_message>
<xml_diff>
--- a/content/W01/D2/demos/C2_W01_D02_decision_tool_STUDENT.xlsx
+++ b/content/W01/D2/demos/C2_W01_D02_decision_tool_STUDENT.xlsx
@@ -722,7 +722,7 @@
         </is>
       </c>
       <c r="B18" s="8">
-        <f>IF(ABS(B10*C6-B6)&gt;=1,"Fix the weekly rate that divides by the wrong weeks before comparing anything.",IF(B13="closed quarters",IF(C7=C5,"Revenue "&amp;IF(B14&lt;0,"fell ","rose ")&amp;TEXT(ABS(B14),"0.0")&amp;" percent"&amp;" between closed quarters of "&amp;C5&amp;" weeks each.","The closed quarters cover different weeks: compare a rate per week."),IF(B13="rate per week","Per week, revenue "&amp;IF(B16&lt;0,"fell ","rose ")&amp;TEXT(ABS(B16),"0.0")&amp;" percent"&amp;" on the cut window.",IF(C6&lt;&gt;C5,"Refuse the comparison: "&amp;C6&amp;" weeks against "&amp;C5&amp;" reads as "&amp;TEXT(ABS(B15),"0.0")&amp;" percent; close the window or use a rate per week.","Revenue "&amp;IF(B15&lt;0,"fell ","rose ")&amp;TEXT(ABS(B15),"0.0")&amp;" percent"&amp;" on matched weeks."))))</f>
+        <f>IF(ABS(B10*C6-B6)&gt;=1,"Fix the weekly rate that divides by the wrong weeks before comparing anything.",IF(B13="closed quarters",IF(C7=C5,"Revenue "&amp;IF(B14&lt;0,"fell ","rose ")&amp;TEXT(ABS(B14),"0.0")&amp;" percent"&amp;" between closed quarters of "&amp;C5&amp;" weeks each.","The closed quarters cover different weeks: compare a rate per week."),IF(B13="rate per week","Per week, revenue "&amp;IF(B16&lt;0,"fell ","rose ")&amp;TEXT(ABS(B16),"0.0")&amp;" percent"&amp;" on the cut window; the rate fixes the length, so send the same weeks of both beside it.",IF(C6&lt;&gt;C5,"Refuse the comparison: "&amp;C6&amp;" weeks against "&amp;C5&amp;" reads as "&amp;TEXT(ABS(B15),"0.0")&amp;" percent; compare the same weeks of both, with a rate per week beside them.","Revenue "&amp;IF(B15&lt;0,"fell ","rose ")&amp;TEXT(ABS(B15),"0.0")&amp;" percent"&amp;" on matched weeks."))))</f>
         <v/>
       </c>
     </row>
@@ -1401,7 +1401,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>The change in orders per customer for every segment, with big moves flagged in their own column rather than dropped.</t>
+          <t>The change in orders per customer for every segment, with big moves flagged in their own column and every segment kept.</t>
         </is>
       </c>
     </row>

</xml_diff>